<commit_message>
Freeroam done + cleanup
</commit_message>
<xml_diff>
--- a/To-Do/MainALR.xlsx
+++ b/To-Do/MainALR.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cmcdonnell1\Downloads\Cost-of-Betrayal\To-Do\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2DED424-23DD-451A-9DC4-552FE162F222}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{97789D77-844A-474A-B3D3-9D4B2488FB0D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="42696" yWindow="144" windowWidth="17880" windowHeight="15348" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="284" uniqueCount="169">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="288" uniqueCount="172">
   <si>
     <t>MainALR</t>
   </si>
@@ -104,18 +104,6 @@
   </si>
   <si>
     <t>To use the sweep scene node to sweep the camera between two locations, put in the first, and current location, in the Scene #1 Slot. It is very important that the camera is already at the first location you input. Next you input the desired location to interpolate to in the Scene #2 Slot, you'll have to tinker a little bit with the speed and rotate value, the rotate value should probably be VERY low though, the default values are about what is good for most cases.</t>
-  </si>
-  <si>
-    <t>Blocked</t>
-  </si>
-  <si>
-    <t>Title Card Popup</t>
-  </si>
-  <si>
-    <t>UI_Popup</t>
-  </si>
-  <si>
-    <t>( TITLE NEEDS TO BE DONE FIRST )  Going to have a popup during in the intro section with a panning camera, this might require some outside UI Design, but honestly it should be something that I can mostly just do inside of Unreal</t>
   </si>
   <si>
     <t>Saving Player Data</t>
@@ -545,6 +533,27 @@
   </si>
   <si>
     <t>A quick time event that'll require the player to spam a button a set amount of times, and if the player doesn't manage to spam it enough, it can lead to an end state, this'll have a customizable amount / resistance based on an integer and/or float value that can be controlled when the node is called</t>
+  </si>
+  <si>
+    <t>Moverment Animation Code</t>
+  </si>
+  <si>
+    <t>BPA_Movement</t>
+  </si>
+  <si>
+    <t>Blocked</t>
+  </si>
+  <si>
+    <t>The animation blueprints responsible for handling animations of the player both in and out of playable sections</t>
+  </si>
+  <si>
+    <t>Intro Credits</t>
+  </si>
+  <si>
+    <t>UI_Credits</t>
+  </si>
+  <si>
+    <t>(FIRST SCENE MUST BE DONE) Introduction credits to pop up during the introduction scenes as we get different views of Carl walking through the desert to El Puente, those scenes must be finished so I can get all the timing right</t>
   </si>
 </sst>
 </file>
@@ -1776,20 +1785,20 @@
     </row>
     <row r="10" spans="1:39" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="D10" s="7" t="s">
-        <v>27</v>
+        <v>167</v>
       </c>
       <c r="E10" s="15" t="s">
-        <v>28</v>
+        <v>169</v>
       </c>
       <c r="F10" s="16"/>
       <c r="G10" s="17"/>
       <c r="H10" s="15" t="s">
-        <v>29</v>
+        <v>170</v>
       </c>
       <c r="I10" s="16"/>
       <c r="J10" s="17"/>
       <c r="K10" s="15" t="s">
-        <v>30</v>
+        <v>171</v>
       </c>
       <c r="L10" s="16"/>
       <c r="M10" s="17"/>
@@ -1824,17 +1833,17 @@
         <v>12</v>
       </c>
       <c r="E11" s="18" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="F11" s="16"/>
       <c r="G11" s="17"/>
       <c r="H11" s="18" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="I11" s="16"/>
       <c r="J11" s="17"/>
       <c r="K11" s="18" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="L11" s="16"/>
       <c r="M11" s="17"/>
@@ -1869,17 +1878,17 @@
         <v>12</v>
       </c>
       <c r="E12" s="15" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="F12" s="16"/>
       <c r="G12" s="17"/>
       <c r="H12" s="15" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="I12" s="16"/>
       <c r="J12" s="17"/>
       <c r="K12" s="15" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="L12" s="16"/>
       <c r="M12" s="17"/>
@@ -1914,17 +1923,17 @@
         <v>12</v>
       </c>
       <c r="E13" s="18" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="F13" s="16"/>
       <c r="G13" s="17"/>
       <c r="H13" s="18" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="I13" s="16"/>
       <c r="J13" s="17"/>
       <c r="K13" s="15" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="L13" s="16"/>
       <c r="M13" s="17"/>
@@ -1959,17 +1968,17 @@
         <v>12</v>
       </c>
       <c r="E14" s="15" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="F14" s="16"/>
       <c r="G14" s="17"/>
       <c r="H14" s="15" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="I14" s="16"/>
       <c r="J14" s="17"/>
       <c r="K14" s="15" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="L14" s="16"/>
       <c r="M14" s="17"/>
@@ -2004,17 +2013,17 @@
         <v>12</v>
       </c>
       <c r="E15" s="18" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="F15" s="16"/>
       <c r="G15" s="17"/>
       <c r="H15" s="19" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="I15" s="16"/>
       <c r="J15" s="17"/>
       <c r="K15" s="19" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="L15" s="16"/>
       <c r="M15" s="17"/>
@@ -2049,17 +2058,17 @@
         <v>12</v>
       </c>
       <c r="E16" s="20" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="F16" s="21"/>
       <c r="G16" s="22"/>
       <c r="H16" s="23" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="I16" s="21"/>
       <c r="J16" s="22"/>
       <c r="K16" s="23" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="L16" s="21"/>
       <c r="M16" s="22"/>
@@ -2094,17 +2103,17 @@
         <v>12</v>
       </c>
       <c r="E17" s="18" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="F17" s="16"/>
       <c r="G17" s="17"/>
       <c r="H17" s="18" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="I17" s="16"/>
       <c r="J17" s="17"/>
       <c r="K17" s="18" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="L17" s="16"/>
       <c r="M17" s="17"/>
@@ -2139,17 +2148,17 @@
         <v>12</v>
       </c>
       <c r="E18" s="15" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="F18" s="16"/>
       <c r="G18" s="17"/>
       <c r="H18" s="15" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="I18" s="16"/>
       <c r="J18" s="17"/>
       <c r="K18" s="15" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="L18" s="16"/>
       <c r="M18" s="17"/>
@@ -2184,17 +2193,17 @@
         <v>12</v>
       </c>
       <c r="E19" s="18" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="F19" s="16"/>
       <c r="G19" s="17"/>
       <c r="H19" s="18" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="I19" s="16"/>
       <c r="J19" s="17"/>
       <c r="K19" s="18" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="L19" s="16"/>
       <c r="M19" s="17"/>
@@ -2229,17 +2238,17 @@
         <v>12</v>
       </c>
       <c r="E20" s="15" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="F20" s="16"/>
       <c r="G20" s="17"/>
       <c r="H20" s="15" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="I20" s="16"/>
       <c r="J20" s="17"/>
       <c r="K20" s="15" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="L20" s="16"/>
       <c r="M20" s="17"/>
@@ -2271,20 +2280,20 @@
     </row>
     <row r="21" spans="4:39" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="D21" s="8" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="E21" s="18" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="F21" s="16"/>
       <c r="G21" s="17"/>
       <c r="H21" s="18" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="I21" s="16"/>
       <c r="J21" s="17"/>
       <c r="K21" s="18" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="L21" s="16"/>
       <c r="M21" s="17"/>
@@ -2319,17 +2328,17 @@
         <v>12</v>
       </c>
       <c r="E22" s="15" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="F22" s="16"/>
       <c r="G22" s="17"/>
       <c r="H22" s="15" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="I22" s="16"/>
       <c r="J22" s="17"/>
       <c r="K22" s="15" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="L22" s="16"/>
       <c r="M22" s="17"/>
@@ -2364,17 +2373,17 @@
         <v>12</v>
       </c>
       <c r="E23" s="18" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="F23" s="16"/>
       <c r="G23" s="17"/>
       <c r="H23" s="18" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="I23" s="16"/>
       <c r="J23" s="17"/>
       <c r="K23" s="18" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="L23" s="16"/>
       <c r="M23" s="17"/>
@@ -2406,20 +2415,20 @@
     </row>
     <row r="24" spans="4:39" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="D24" s="7" t="s">
-        <v>61</v>
+        <v>12</v>
       </c>
       <c r="E24" s="15" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="F24" s="16"/>
       <c r="G24" s="17"/>
       <c r="H24" s="24" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="I24" s="16"/>
       <c r="J24" s="17"/>
       <c r="K24" s="24" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="L24" s="16"/>
       <c r="M24" s="17"/>
@@ -2454,17 +2463,17 @@
         <v>12</v>
       </c>
       <c r="E25" s="18" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="F25" s="16"/>
       <c r="G25" s="17"/>
       <c r="H25" s="19" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="I25" s="16"/>
       <c r="J25" s="17"/>
       <c r="K25" s="19" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="L25" s="16"/>
       <c r="M25" s="17"/>
@@ -2499,17 +2508,17 @@
         <v>12</v>
       </c>
       <c r="E26" s="15" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="F26" s="16"/>
       <c r="G26" s="17"/>
       <c r="H26" s="15" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="I26" s="16"/>
       <c r="J26" s="17"/>
       <c r="K26" s="15" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="L26" s="16"/>
       <c r="M26" s="17"/>
@@ -2544,17 +2553,17 @@
         <v>12</v>
       </c>
       <c r="E27" s="18" t="s">
-        <v>166</v>
+        <v>162</v>
       </c>
       <c r="F27" s="16"/>
       <c r="G27" s="17"/>
       <c r="H27" s="18" t="s">
-        <v>167</v>
+        <v>163</v>
       </c>
       <c r="I27" s="16"/>
       <c r="J27" s="17"/>
       <c r="K27" s="18" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="L27" s="16"/>
       <c r="M27" s="17"/>
@@ -2585,14 +2594,22 @@
       <c r="AM27" s="17"/>
     </row>
     <row r="28" spans="4:39" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="D28" s="7"/>
-      <c r="E28" s="15"/>
+      <c r="D28" s="7" t="s">
+        <v>167</v>
+      </c>
+      <c r="E28" s="15" t="s">
+        <v>165</v>
+      </c>
       <c r="F28" s="16"/>
       <c r="G28" s="17"/>
-      <c r="H28" s="15"/>
+      <c r="H28" s="15" t="s">
+        <v>166</v>
+      </c>
       <c r="I28" s="16"/>
       <c r="J28" s="17"/>
-      <c r="K28" s="15"/>
+      <c r="K28" s="15" t="s">
+        <v>168</v>
+      </c>
       <c r="L28" s="16"/>
       <c r="M28" s="17"/>
       <c r="N28" s="2"/>
@@ -6866,10 +6883,10 @@
   <sheetData>
     <row r="1" spans="1:44" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="E1" s="2"/>
       <c r="F1" s="2"/>
@@ -6877,7 +6894,7 @@
     <row r="2" spans="1:44" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="3" spans="1:44" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="D3" s="1" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="E3" s="3"/>
     </row>
@@ -6907,7 +6924,7 @@
         <v>7</v>
       </c>
       <c r="E5" s="32" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="F5" s="16"/>
       <c r="G5" s="17"/>
@@ -6922,7 +6939,7 @@
       <c r="L5" s="16"/>
       <c r="M5" s="17"/>
       <c r="N5" s="32" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="O5" s="16"/>
       <c r="P5" s="17"/>
@@ -6931,7 +6948,7 @@
         <v>7</v>
       </c>
       <c r="S5" s="32" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="T5" s="16"/>
       <c r="U5" s="17"/>
@@ -6946,7 +6963,7 @@
       <c r="Z5" s="16"/>
       <c r="AA5" s="17"/>
       <c r="AB5" s="32" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="AC5" s="16"/>
       <c r="AD5" s="17"/>
@@ -6954,7 +6971,7 @@
         <v>7</v>
       </c>
       <c r="AG5" s="37" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="AH5" s="21"/>
       <c r="AI5" s="22"/>
@@ -6969,7 +6986,7 @@
       <c r="AN5" s="16"/>
       <c r="AO5" s="17"/>
       <c r="AP5" s="32" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="AQ5" s="16"/>
       <c r="AR5" s="17"/>
@@ -6983,17 +7000,17 @@
         <v>12</v>
       </c>
       <c r="E6" s="15" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="F6" s="16"/>
       <c r="G6" s="17"/>
       <c r="H6" s="15" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="I6" s="16"/>
       <c r="J6" s="17"/>
       <c r="K6" s="15" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="L6" s="16"/>
       <c r="M6" s="17"/>
@@ -7037,17 +7054,17 @@
         <v>12</v>
       </c>
       <c r="E7" s="18" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="F7" s="16"/>
       <c r="G7" s="17"/>
       <c r="H7" s="18" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="I7" s="16"/>
       <c r="J7" s="17"/>
       <c r="K7" s="18" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="L7" s="16"/>
       <c r="M7" s="17"/>
@@ -7089,17 +7106,17 @@
       <c r="B8" s="17"/>
       <c r="D8" s="7"/>
       <c r="E8" s="15" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="F8" s="16"/>
       <c r="G8" s="17"/>
       <c r="H8" s="18" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="I8" s="16"/>
       <c r="J8" s="17"/>
       <c r="K8" s="15" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="L8" s="16"/>
       <c r="M8" s="17"/>
@@ -7137,17 +7154,17 @@
     <row r="9" spans="1:44" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="D9" s="7"/>
       <c r="E9" s="18" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="F9" s="16"/>
       <c r="G9" s="17"/>
       <c r="H9" s="18" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="I9" s="16"/>
       <c r="J9" s="17"/>
       <c r="K9" s="18" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="L9" s="16"/>
       <c r="M9" s="17"/>
@@ -7185,17 +7202,17 @@
     <row r="10" spans="1:44" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="D10" s="7"/>
       <c r="E10" s="15" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="F10" s="16"/>
       <c r="G10" s="17"/>
       <c r="H10" s="18" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="I10" s="16"/>
       <c r="J10" s="17"/>
       <c r="K10" s="15" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="L10" s="16"/>
       <c r="M10" s="17"/>
@@ -7232,22 +7249,22 @@
     </row>
     <row r="11" spans="1:44" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="3" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="B11" s="3"/>
       <c r="D11" s="7"/>
       <c r="E11" s="18" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="F11" s="16"/>
       <c r="G11" s="17"/>
       <c r="H11" s="18" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="I11" s="16"/>
       <c r="J11" s="17"/>
       <c r="K11" s="18" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="L11" s="16"/>
       <c r="M11" s="17"/>
@@ -7285,17 +7302,17 @@
     <row r="12" spans="1:44" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="D12" s="7"/>
       <c r="E12" s="15" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="F12" s="16"/>
       <c r="G12" s="17"/>
       <c r="H12" s="18" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="I12" s="16"/>
       <c r="J12" s="17"/>
       <c r="K12" s="15" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="L12" s="16"/>
       <c r="M12" s="17"/>
@@ -7335,17 +7352,17 @@
         <v>12</v>
       </c>
       <c r="E13" s="18" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="F13" s="16"/>
       <c r="G13" s="17"/>
       <c r="H13" s="18" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="I13" s="16"/>
       <c r="J13" s="17"/>
       <c r="K13" s="18" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="L13" s="16"/>
       <c r="M13" s="17"/>
@@ -7383,17 +7400,17 @@
     <row r="14" spans="1:44" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="D14" s="7"/>
       <c r="E14" s="15" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="F14" s="16"/>
       <c r="G14" s="17"/>
       <c r="H14" s="15" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="I14" s="16"/>
       <c r="J14" s="17"/>
       <c r="K14" s="15" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="L14" s="16"/>
       <c r="M14" s="17"/>
@@ -7430,24 +7447,24 @@
     </row>
     <row r="15" spans="1:44" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="3" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="B15" s="3"/>
       <c r="D15" s="7" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="E15" s="18" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="F15" s="16"/>
       <c r="G15" s="17"/>
       <c r="H15" s="18" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="I15" s="16"/>
       <c r="J15" s="17"/>
       <c r="K15" s="18" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="L15" s="16"/>
       <c r="M15" s="17"/>
@@ -12097,10 +12114,10 @@
   <sheetData>
     <row r="1" spans="1:44" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="E1" s="2"/>
       <c r="F1" s="2"/>
@@ -12108,7 +12125,7 @@
     <row r="2" spans="1:44" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="3" spans="1:44" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="D3" s="1" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="E3" s="3"/>
     </row>
@@ -12138,7 +12155,7 @@
         <v>7</v>
       </c>
       <c r="E5" s="32" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="F5" s="16"/>
       <c r="G5" s="17"/>
@@ -12153,7 +12170,7 @@
       <c r="L5" s="16"/>
       <c r="M5" s="17"/>
       <c r="N5" s="32" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="O5" s="16"/>
       <c r="P5" s="17"/>
@@ -12162,7 +12179,7 @@
         <v>7</v>
       </c>
       <c r="S5" s="32" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="T5" s="16"/>
       <c r="U5" s="17"/>
@@ -12177,7 +12194,7 @@
       <c r="Z5" s="16"/>
       <c r="AA5" s="17"/>
       <c r="AB5" s="32" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="AC5" s="16"/>
       <c r="AD5" s="17"/>
@@ -12185,7 +12202,7 @@
         <v>7</v>
       </c>
       <c r="AG5" s="37" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="AH5" s="21"/>
       <c r="AI5" s="22"/>
@@ -12200,36 +12217,36 @@
       <c r="AN5" s="16"/>
       <c r="AO5" s="17"/>
       <c r="AP5" s="32" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="AQ5" s="16"/>
       <c r="AR5" s="17"/>
     </row>
     <row r="6" spans="1:44" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="35" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="B6" s="17"/>
       <c r="D6" s="7" t="s">
         <v>12</v>
       </c>
       <c r="E6" s="39" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="F6" s="16"/>
       <c r="G6" s="17"/>
       <c r="H6" s="15" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="I6" s="16"/>
       <c r="J6" s="17"/>
       <c r="K6" s="15" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="L6" s="16"/>
       <c r="M6" s="17"/>
       <c r="N6" s="15" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="O6" s="16"/>
       <c r="P6" s="17"/>
@@ -12263,27 +12280,27 @@
     </row>
     <row r="7" spans="1:44" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="35" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="B7" s="17"/>
       <c r="D7" s="7"/>
       <c r="E7" s="40" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="F7" s="16"/>
       <c r="G7" s="17"/>
       <c r="H7" s="18" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="I7" s="16"/>
       <c r="J7" s="17"/>
       <c r="K7" s="18" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="L7" s="16"/>
       <c r="M7" s="17"/>
       <c r="N7" s="18" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="O7" s="16"/>
       <c r="P7" s="17"/>
@@ -12317,29 +12334,29 @@
     </row>
     <row r="8" spans="1:44" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="35" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="B8" s="17"/>
       <c r="D8" s="7" t="s">
         <v>12</v>
       </c>
       <c r="E8" s="39" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="F8" s="16"/>
       <c r="G8" s="17"/>
       <c r="H8" s="15" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="I8" s="16"/>
       <c r="J8" s="17"/>
       <c r="K8" s="15" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="L8" s="16"/>
       <c r="M8" s="17"/>
       <c r="N8" s="15" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="O8" s="16"/>
       <c r="P8" s="17"/>
@@ -12374,22 +12391,22 @@
     <row r="9" spans="1:44" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="D9" s="7"/>
       <c r="E9" s="18" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="F9" s="16"/>
       <c r="G9" s="17"/>
       <c r="H9" s="18" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="I9" s="16"/>
       <c r="J9" s="17"/>
       <c r="K9" s="18" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="L9" s="16"/>
       <c r="M9" s="17"/>
       <c r="N9" s="38" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="O9" s="16"/>
       <c r="P9" s="17"/>
@@ -12424,22 +12441,22 @@
     <row r="10" spans="1:44" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="D10" s="7"/>
       <c r="E10" s="15" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="F10" s="16"/>
       <c r="G10" s="17"/>
       <c r="H10" s="15" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="I10" s="16"/>
       <c r="J10" s="17"/>
       <c r="K10" s="15" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="L10" s="16"/>
       <c r="M10" s="17"/>
       <c r="N10" s="15" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="O10" s="16"/>
       <c r="P10" s="17"/>
@@ -12473,24 +12490,24 @@
     </row>
     <row r="11" spans="1:44" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="3" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="B11" s="3"/>
       <c r="D11" s="7" t="s">
         <v>12</v>
       </c>
       <c r="E11" s="18" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="F11" s="16"/>
       <c r="G11" s="17"/>
       <c r="H11" s="18" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="I11" s="16"/>
       <c r="J11" s="17"/>
       <c r="K11" s="18" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="L11" s="16"/>
       <c r="M11" s="17"/>
@@ -12528,22 +12545,22 @@
     <row r="12" spans="1:44" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="D12" s="7"/>
       <c r="E12" s="15" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="F12" s="16"/>
       <c r="G12" s="17"/>
       <c r="H12" s="15" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
       <c r="I12" s="16"/>
       <c r="J12" s="17"/>
       <c r="K12" s="15" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="L12" s="16"/>
       <c r="M12" s="17"/>
       <c r="N12" s="41" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="O12" s="16"/>
       <c r="P12" s="17"/>
@@ -12578,22 +12595,22 @@
     <row r="13" spans="1:44" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="D13" s="7"/>
       <c r="E13" s="18" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="F13" s="16"/>
       <c r="G13" s="17"/>
       <c r="H13" s="18" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="I13" s="16"/>
       <c r="J13" s="17"/>
       <c r="K13" s="18" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="L13" s="16"/>
       <c r="M13" s="17"/>
       <c r="N13" s="38" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="O13" s="16"/>
       <c r="P13" s="17"/>
@@ -12630,22 +12647,22 @@
         <v>12</v>
       </c>
       <c r="E14" s="15" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
       <c r="F14" s="16"/>
       <c r="G14" s="17"/>
       <c r="H14" s="15" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
       <c r="I14" s="16"/>
       <c r="J14" s="17"/>
       <c r="K14" s="15" t="s">
-        <v>145</v>
+        <v>141</v>
       </c>
       <c r="L14" s="16"/>
       <c r="M14" s="17"/>
       <c r="N14" s="42" t="s">
-        <v>146</v>
+        <v>142</v>
       </c>
       <c r="O14" s="16"/>
       <c r="P14" s="17"/>
@@ -12679,24 +12696,24 @@
     </row>
     <row r="15" spans="1:44" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="3" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="B15" s="3"/>
       <c r="D15" s="7" t="s">
         <v>12</v>
       </c>
       <c r="E15" s="18" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="F15" s="16"/>
       <c r="G15" s="17"/>
       <c r="H15" s="18" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="I15" s="16"/>
       <c r="J15" s="17"/>
       <c r="K15" s="18" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="L15" s="16"/>
       <c r="M15" s="17"/>
@@ -17352,10 +17369,10 @@
   <sheetData>
     <row r="1" spans="1:44" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
       <c r="E1" s="2"/>
       <c r="F1" s="2"/>
@@ -17363,7 +17380,7 @@
     <row r="2" spans="1:44" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="3" spans="1:44" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="D3" s="1" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="E3" s="3"/>
     </row>
@@ -17393,7 +17410,7 @@
         <v>7</v>
       </c>
       <c r="E5" s="32" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="F5" s="16"/>
       <c r="G5" s="17"/>
@@ -17408,7 +17425,7 @@
       <c r="L5" s="16"/>
       <c r="M5" s="17"/>
       <c r="N5" s="32" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="O5" s="16"/>
       <c r="P5" s="17"/>
@@ -17417,7 +17434,7 @@
         <v>7</v>
       </c>
       <c r="S5" s="32" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="T5" s="16"/>
       <c r="U5" s="17"/>
@@ -17432,7 +17449,7 @@
       <c r="Z5" s="16"/>
       <c r="AA5" s="17"/>
       <c r="AB5" s="32" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="AC5" s="16"/>
       <c r="AD5" s="17"/>
@@ -17440,7 +17457,7 @@
         <v>7</v>
       </c>
       <c r="AG5" s="37" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="AH5" s="21"/>
       <c r="AI5" s="22"/>
@@ -17455,7 +17472,7 @@
       <c r="AN5" s="16"/>
       <c r="AO5" s="17"/>
       <c r="AP5" s="32" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="AQ5" s="16"/>
       <c r="AR5" s="17"/>
@@ -17469,17 +17486,17 @@
         <v>12</v>
       </c>
       <c r="E6" s="15" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="F6" s="16"/>
       <c r="G6" s="17"/>
       <c r="H6" s="15" t="s">
-        <v>152</v>
+        <v>148</v>
       </c>
       <c r="I6" s="16"/>
       <c r="J6" s="17"/>
       <c r="K6" s="15" t="s">
-        <v>153</v>
+        <v>149</v>
       </c>
       <c r="L6" s="16"/>
       <c r="M6" s="17"/>
@@ -17521,17 +17538,17 @@
       <c r="B7" s="17"/>
       <c r="D7" s="7"/>
       <c r="E7" s="18" t="s">
-        <v>154</v>
+        <v>150</v>
       </c>
       <c r="F7" s="16"/>
       <c r="G7" s="17"/>
       <c r="H7" s="18" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="I7" s="16"/>
       <c r="J7" s="17"/>
       <c r="K7" s="18" t="s">
-        <v>156</v>
+        <v>152</v>
       </c>
       <c r="L7" s="16"/>
       <c r="M7" s="17"/>
@@ -17573,17 +17590,17 @@
       <c r="B8" s="17"/>
       <c r="D8" s="7"/>
       <c r="E8" s="15" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="F8" s="16"/>
       <c r="G8" s="17"/>
       <c r="H8" s="15" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
       <c r="I8" s="16"/>
       <c r="J8" s="17"/>
       <c r="K8" s="15" t="s">
-        <v>159</v>
+        <v>155</v>
       </c>
       <c r="L8" s="16"/>
       <c r="M8" s="17"/>
@@ -17621,17 +17638,17 @@
     <row r="9" spans="1:44" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="D9" s="7"/>
       <c r="E9" s="18" t="s">
-        <v>160</v>
+        <v>156</v>
       </c>
       <c r="F9" s="16"/>
       <c r="G9" s="17"/>
       <c r="H9" s="18" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
       <c r="I9" s="16"/>
       <c r="J9" s="17"/>
       <c r="K9" s="18" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="L9" s="16"/>
       <c r="M9" s="17"/>
@@ -17669,17 +17686,17 @@
     <row r="10" spans="1:44" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="D10" s="7"/>
       <c r="E10" s="15" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
       <c r="F10" s="16"/>
       <c r="G10" s="17"/>
       <c r="H10" s="15" t="s">
-        <v>164</v>
+        <v>160</v>
       </c>
       <c r="I10" s="16"/>
       <c r="J10" s="17"/>
       <c r="K10" s="15" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
       <c r="L10" s="16"/>
       <c r="M10" s="17"/>
@@ -17716,7 +17733,7 @@
     </row>
     <row r="11" spans="1:44" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="3" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="B11" s="3"/>
       <c r="D11" s="7"/>
@@ -17888,7 +17905,7 @@
     </row>
     <row r="15" spans="1:44" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="3" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="B15" s="3"/>
       <c r="D15" s="7"/>

</xml_diff>

<commit_message>
Terrain Work + edits
</commit_message>
<xml_diff>
--- a/To-Do/MainALR.xlsx
+++ b/To-Do/MainALR.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cmcdonnell1\Downloads\Cost-of-Betrayal\To-Do\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4A08460-A7E1-49A6-9150-5F4AF7E156AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1BDA60FC-1116-4045-963C-156A1A8E862C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="42696" yWindow="144" windowWidth="17880" windowHeight="15348" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="42696" yWindow="144" windowWidth="17880" windowHeight="15348" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Coding" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="307" uniqueCount="183">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="308" uniqueCount="183">
   <si>
     <t>MainALR</t>
   </si>
@@ -229,9 +229,6 @@
     <t>Node Name: Begin Freeroam</t>
   </si>
   <si>
-    <t>A node that'll allow developers to switch from a regular scene to one in witch the player has complete control of the movement of the character and can interact with the background and area around them</t>
-  </si>
-  <si>
     <t>Screen Shakeing</t>
   </si>
   <si>
@@ -302,12 +299,6 @@
   </si>
   <si>
     <t xml:space="preserve"> </t>
-  </si>
-  <si>
-    <t>El Puente  Rocky Terrain</t>
-  </si>
-  <si>
-    <t>terrain bro, mostly flat for the town</t>
   </si>
   <si>
     <t>Tumbleweed Model</t>
@@ -587,6 +578,15 @@
   </si>
   <si>
     <t>A blueprint that can allow multiple meshes to be combined into a single model for use in the game up to 6 meshes at once.</t>
+  </si>
+  <si>
+    <t>A node that allows developers to switch from a regular scene to one in which the player has complete control of the movement of the character and can interact with the background and area around them</t>
+  </si>
+  <si>
+    <t>El Puente Props</t>
+  </si>
+  <si>
+    <t>props such as fences, chairs, benches, crates, barrels, a centerpiece for the town, hitching posts, and lanturns. (feel free to add any other shit u come up with too)</t>
   </si>
 </sst>
 </file>
@@ -1830,20 +1830,20 @@
     </row>
     <row r="10" spans="1:39" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="D10" s="7" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="E10" s="15" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="F10" s="16"/>
       <c r="G10" s="17"/>
       <c r="H10" s="15" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="I10" s="16"/>
       <c r="J10" s="17"/>
       <c r="K10" s="15" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="L10" s="16"/>
       <c r="M10" s="17"/>
@@ -2473,7 +2473,7 @@
       <c r="I24" s="16"/>
       <c r="J24" s="17"/>
       <c r="K24" s="18" t="s">
-        <v>68</v>
+        <v>180</v>
       </c>
       <c r="L24" s="16"/>
       <c r="M24" s="17"/>
@@ -2508,17 +2508,17 @@
         <v>12</v>
       </c>
       <c r="E25" s="25" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F25" s="16"/>
       <c r="G25" s="17"/>
       <c r="H25" s="26" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="I25" s="16"/>
       <c r="J25" s="17"/>
       <c r="K25" s="26" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="L25" s="16"/>
       <c r="M25" s="17"/>
@@ -2553,17 +2553,17 @@
         <v>12</v>
       </c>
       <c r="E26" s="15" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="F26" s="16"/>
       <c r="G26" s="17"/>
       <c r="H26" s="15" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="I26" s="16"/>
       <c r="J26" s="17"/>
       <c r="K26" s="15" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="L26" s="16"/>
       <c r="M26" s="17"/>
@@ -2598,17 +2598,17 @@
         <v>12</v>
       </c>
       <c r="E27" s="25" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="F27" s="16"/>
       <c r="G27" s="17"/>
       <c r="H27" s="25" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="I27" s="16"/>
       <c r="J27" s="17"/>
       <c r="K27" s="25" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="L27" s="16"/>
       <c r="M27" s="17"/>
@@ -2640,20 +2640,20 @@
     </row>
     <row r="28" spans="4:39" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="D28" s="7" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="E28" s="15" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="F28" s="16"/>
       <c r="G28" s="17"/>
       <c r="H28" s="15" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="I28" s="16"/>
       <c r="J28" s="17"/>
       <c r="K28" s="15" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="L28" s="16"/>
       <c r="M28" s="17"/>
@@ -2688,17 +2688,17 @@
         <v>12</v>
       </c>
       <c r="E29" s="25" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="F29" s="16"/>
       <c r="G29" s="17"/>
       <c r="H29" s="25" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="I29" s="16"/>
       <c r="J29" s="17"/>
       <c r="K29" s="25" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="L29" s="16"/>
       <c r="M29" s="17"/>
@@ -2731,17 +2731,17 @@
     <row r="30" spans="4:39" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="D30" s="7"/>
       <c r="E30" s="15" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="F30" s="16"/>
       <c r="G30" s="17"/>
       <c r="H30" s="15" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="I30" s="16"/>
       <c r="J30" s="17"/>
       <c r="K30" s="15" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="L30" s="16"/>
       <c r="M30" s="17"/>
@@ -2776,17 +2776,17 @@
         <v>12</v>
       </c>
       <c r="E31" s="25" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="F31" s="16"/>
       <c r="G31" s="17"/>
       <c r="H31" s="25" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="I31" s="16"/>
       <c r="J31" s="17"/>
       <c r="K31" s="25" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="L31" s="16"/>
       <c r="M31" s="17"/>
@@ -2821,17 +2821,17 @@
         <v>12</v>
       </c>
       <c r="E32" s="15" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="F32" s="16"/>
       <c r="G32" s="17"/>
       <c r="H32" s="15" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
       <c r="I32" s="16"/>
       <c r="J32" s="17"/>
       <c r="K32" s="15" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="L32" s="16"/>
       <c r="M32" s="17"/>
@@ -6958,10 +6958,10 @@
   <sheetData>
     <row r="1" spans="1:44" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>75</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>76</v>
       </c>
       <c r="E1" s="2"/>
       <c r="F1" s="2"/>
@@ -6969,7 +6969,7 @@
     <row r="2" spans="1:44" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="3" spans="1:44" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="D3" s="1" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="E3" s="3"/>
     </row>
@@ -6999,7 +6999,7 @@
         <v>7</v>
       </c>
       <c r="E5" s="31" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="F5" s="16"/>
       <c r="G5" s="17"/>
@@ -7014,7 +7014,7 @@
       <c r="L5" s="16"/>
       <c r="M5" s="17"/>
       <c r="N5" s="31" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="O5" s="16"/>
       <c r="P5" s="17"/>
@@ -7023,7 +7023,7 @@
         <v>7</v>
       </c>
       <c r="S5" s="31" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="T5" s="16"/>
       <c r="U5" s="17"/>
@@ -7038,7 +7038,7 @@
       <c r="Z5" s="16"/>
       <c r="AA5" s="17"/>
       <c r="AB5" s="31" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="AC5" s="16"/>
       <c r="AD5" s="17"/>
@@ -7046,7 +7046,7 @@
         <v>7</v>
       </c>
       <c r="AG5" s="36" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="AH5" s="20"/>
       <c r="AI5" s="21"/>
@@ -7061,7 +7061,7 @@
       <c r="AN5" s="16"/>
       <c r="AO5" s="17"/>
       <c r="AP5" s="31" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="AQ5" s="16"/>
       <c r="AR5" s="17"/>
@@ -7075,17 +7075,17 @@
         <v>12</v>
       </c>
       <c r="E6" s="15" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="F6" s="16"/>
       <c r="G6" s="17"/>
       <c r="H6" s="15" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="I6" s="16"/>
       <c r="J6" s="17"/>
       <c r="K6" s="15" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="L6" s="16"/>
       <c r="M6" s="17"/>
@@ -7129,17 +7129,17 @@
         <v>12</v>
       </c>
       <c r="E7" s="25" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="F7" s="16"/>
       <c r="G7" s="17"/>
       <c r="H7" s="25" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="I7" s="16"/>
       <c r="J7" s="17"/>
       <c r="K7" s="25" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="L7" s="16"/>
       <c r="M7" s="17"/>
@@ -7181,17 +7181,17 @@
       <c r="B8" s="17"/>
       <c r="D8" s="7"/>
       <c r="E8" s="15" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="F8" s="16"/>
       <c r="G8" s="17"/>
       <c r="H8" s="25" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="I8" s="16"/>
       <c r="J8" s="17"/>
       <c r="K8" s="15" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="L8" s="16"/>
       <c r="M8" s="17"/>
@@ -7229,17 +7229,17 @@
     <row r="9" spans="1:44" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="D9" s="7"/>
       <c r="E9" s="25" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="F9" s="16"/>
       <c r="G9" s="17"/>
       <c r="H9" s="25" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="I9" s="16"/>
       <c r="J9" s="17"/>
       <c r="K9" s="25" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="L9" s="16"/>
       <c r="M9" s="17"/>
@@ -7277,17 +7277,17 @@
     <row r="10" spans="1:44" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="D10" s="7"/>
       <c r="E10" s="15" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="F10" s="16"/>
       <c r="G10" s="17"/>
       <c r="H10" s="25" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="I10" s="16"/>
       <c r="J10" s="17"/>
       <c r="K10" s="15" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="L10" s="16"/>
       <c r="M10" s="17"/>
@@ -7324,22 +7324,22 @@
     </row>
     <row r="11" spans="1:44" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="3" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B11" s="3"/>
       <c r="D11" s="7"/>
       <c r="E11" s="25" t="s">
-        <v>93</v>
+        <v>181</v>
       </c>
       <c r="F11" s="16"/>
       <c r="G11" s="17"/>
       <c r="H11" s="25" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="I11" s="16"/>
       <c r="J11" s="17"/>
       <c r="K11" s="25" t="s">
-        <v>94</v>
+        <v>182</v>
       </c>
       <c r="L11" s="16"/>
       <c r="M11" s="17"/>
@@ -7377,17 +7377,17 @@
     <row r="12" spans="1:44" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="D12" s="7"/>
       <c r="E12" s="15" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="F12" s="16"/>
       <c r="G12" s="17"/>
       <c r="H12" s="25" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="I12" s="16"/>
       <c r="J12" s="17"/>
       <c r="K12" s="15" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="L12" s="16"/>
       <c r="M12" s="17"/>
@@ -7427,17 +7427,17 @@
         <v>12</v>
       </c>
       <c r="E13" s="25" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="F13" s="16"/>
       <c r="G13" s="17"/>
       <c r="H13" s="25" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="I13" s="16"/>
       <c r="J13" s="17"/>
       <c r="K13" s="25" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="L13" s="16"/>
       <c r="M13" s="17"/>
@@ -7473,19 +7473,21 @@
       <c r="AR13" s="17"/>
     </row>
     <row r="14" spans="1:44" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="D14" s="7"/>
+      <c r="D14" s="7" t="s">
+        <v>12</v>
+      </c>
       <c r="E14" s="15" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="F14" s="16"/>
       <c r="G14" s="17"/>
       <c r="H14" s="15" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="I14" s="16"/>
       <c r="J14" s="17"/>
       <c r="K14" s="15" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="L14" s="16"/>
       <c r="M14" s="17"/>
@@ -7522,24 +7524,24 @@
     </row>
     <row r="15" spans="1:44" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="3" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B15" s="3"/>
       <c r="D15" s="7" t="s">
-        <v>57</v>
+        <v>12</v>
       </c>
       <c r="E15" s="25" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="F15" s="16"/>
       <c r="G15" s="17"/>
       <c r="H15" s="25" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="I15" s="16"/>
       <c r="J15" s="17"/>
       <c r="K15" s="25" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="L15" s="16"/>
       <c r="M15" s="17"/>
@@ -12189,10 +12191,10 @@
   <sheetData>
     <row r="1" spans="1:44" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="E1" s="2"/>
       <c r="F1" s="2"/>
@@ -12200,7 +12202,7 @@
     <row r="2" spans="1:44" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="3" spans="1:44" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="D3" s="1" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="E3" s="3"/>
     </row>
@@ -12230,7 +12232,7 @@
         <v>7</v>
       </c>
       <c r="E5" s="31" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="F5" s="16"/>
       <c r="G5" s="17"/>
@@ -12245,7 +12247,7 @@
       <c r="L5" s="16"/>
       <c r="M5" s="17"/>
       <c r="N5" s="31" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="O5" s="16"/>
       <c r="P5" s="17"/>
@@ -12254,7 +12256,7 @@
         <v>7</v>
       </c>
       <c r="S5" s="31" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="T5" s="16"/>
       <c r="U5" s="17"/>
@@ -12269,7 +12271,7 @@
       <c r="Z5" s="16"/>
       <c r="AA5" s="17"/>
       <c r="AB5" s="31" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="AC5" s="16"/>
       <c r="AD5" s="17"/>
@@ -12277,7 +12279,7 @@
         <v>7</v>
       </c>
       <c r="AG5" s="36" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="AH5" s="20"/>
       <c r="AI5" s="21"/>
@@ -12292,36 +12294,36 @@
       <c r="AN5" s="16"/>
       <c r="AO5" s="17"/>
       <c r="AP5" s="31" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="AQ5" s="16"/>
       <c r="AR5" s="17"/>
     </row>
     <row r="6" spans="1:44" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="29" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="B6" s="17"/>
       <c r="D6" s="7" t="s">
         <v>12</v>
       </c>
       <c r="E6" s="43" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="F6" s="16"/>
       <c r="G6" s="17"/>
       <c r="H6" s="15" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="I6" s="16"/>
       <c r="J6" s="17"/>
       <c r="K6" s="15" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="L6" s="16"/>
       <c r="M6" s="17"/>
       <c r="N6" s="15" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="O6" s="16"/>
       <c r="P6" s="17"/>
@@ -12355,29 +12357,29 @@
     </row>
     <row r="7" spans="1:44" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="29" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="B7" s="17"/>
       <c r="D7" s="7" t="s">
         <v>12</v>
       </c>
       <c r="E7" s="44" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="F7" s="16"/>
       <c r="G7" s="17"/>
       <c r="H7" s="25" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="I7" s="16"/>
       <c r="J7" s="17"/>
       <c r="K7" s="25" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="L7" s="16"/>
       <c r="M7" s="17"/>
       <c r="N7" s="25" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="O7" s="16"/>
       <c r="P7" s="17"/>
@@ -12411,14 +12413,14 @@
     </row>
     <row r="8" spans="1:44" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="29" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="B8" s="17"/>
       <c r="D8" s="7" t="s">
         <v>12</v>
       </c>
       <c r="E8" s="43" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="F8" s="16"/>
       <c r="G8" s="17"/>
@@ -12428,12 +12430,12 @@
       <c r="I8" s="16"/>
       <c r="J8" s="17"/>
       <c r="K8" s="15" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="L8" s="16"/>
       <c r="M8" s="17"/>
       <c r="N8" s="15" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="O8" s="16"/>
       <c r="P8" s="17"/>
@@ -12468,22 +12470,22 @@
     <row r="9" spans="1:44" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="D9" s="7"/>
       <c r="E9" s="25" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="F9" s="16"/>
       <c r="G9" s="17"/>
       <c r="H9" s="25" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="I9" s="16"/>
       <c r="J9" s="17"/>
       <c r="K9" s="25" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="L9" s="16"/>
       <c r="M9" s="17"/>
       <c r="N9" s="38" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="O9" s="16"/>
       <c r="P9" s="17"/>
@@ -12517,25 +12519,25 @@
     </row>
     <row r="10" spans="1:44" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="D10" s="7" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="E10" s="15" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="F10" s="16"/>
       <c r="G10" s="17"/>
       <c r="H10" s="15" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="I10" s="16"/>
       <c r="J10" s="17"/>
       <c r="K10" s="15" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="L10" s="16"/>
       <c r="M10" s="17"/>
       <c r="N10" s="45" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
       <c r="O10" s="16"/>
       <c r="P10" s="17"/>
@@ -12569,24 +12571,24 @@
     </row>
     <row r="11" spans="1:44" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="3" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B11" s="3"/>
       <c r="D11" s="7" t="s">
         <v>12</v>
       </c>
       <c r="E11" s="25" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="F11" s="16"/>
       <c r="G11" s="17"/>
       <c r="H11" s="25" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="I11" s="16"/>
       <c r="J11" s="17"/>
       <c r="K11" s="25" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="L11" s="16"/>
       <c r="M11" s="17"/>
@@ -12626,22 +12628,22 @@
         <v>12</v>
       </c>
       <c r="E12" s="15" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="F12" s="16"/>
       <c r="G12" s="17"/>
       <c r="H12" s="15" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="I12" s="16"/>
       <c r="J12" s="17"/>
       <c r="K12" s="15" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="L12" s="16"/>
       <c r="M12" s="17"/>
       <c r="N12" s="42" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="O12" s="16"/>
       <c r="P12" s="17"/>
@@ -12678,22 +12680,22 @@
         <v>12</v>
       </c>
       <c r="E13" s="25" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="F13" s="16"/>
       <c r="G13" s="17"/>
       <c r="H13" s="25" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="I13" s="16"/>
       <c r="J13" s="17"/>
       <c r="K13" s="25" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="L13" s="16"/>
       <c r="M13" s="17"/>
       <c r="N13" s="38" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="O13" s="16"/>
       <c r="P13" s="17"/>
@@ -12730,22 +12732,22 @@
         <v>12</v>
       </c>
       <c r="E14" s="15" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="F14" s="16"/>
       <c r="G14" s="17"/>
       <c r="H14" s="15" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="I14" s="16"/>
       <c r="J14" s="17"/>
       <c r="K14" s="15" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="L14" s="16"/>
       <c r="M14" s="17"/>
       <c r="N14" s="39" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="O14" s="16"/>
       <c r="P14" s="17"/>
@@ -12779,14 +12781,14 @@
     </row>
     <row r="15" spans="1:44" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="3" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B15" s="3"/>
       <c r="D15" s="7" t="s">
         <v>12</v>
       </c>
       <c r="E15" s="25" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="F15" s="16"/>
       <c r="G15" s="17"/>
@@ -12796,7 +12798,7 @@
       <c r="I15" s="16"/>
       <c r="J15" s="17"/>
       <c r="K15" s="25" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="L15" s="16"/>
       <c r="M15" s="17"/>
@@ -17453,10 +17455,10 @@
   <sheetData>
     <row r="1" spans="1:44" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="E1" s="2"/>
       <c r="F1" s="2"/>
@@ -17464,7 +17466,7 @@
     <row r="2" spans="1:44" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="3" spans="1:44" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="D3" s="1" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="E3" s="3"/>
     </row>
@@ -17494,7 +17496,7 @@
         <v>7</v>
       </c>
       <c r="E5" s="31" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="F5" s="16"/>
       <c r="G5" s="17"/>
@@ -17509,7 +17511,7 @@
       <c r="L5" s="16"/>
       <c r="M5" s="17"/>
       <c r="N5" s="31" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="O5" s="16"/>
       <c r="P5" s="17"/>
@@ -17518,7 +17520,7 @@
         <v>7</v>
       </c>
       <c r="S5" s="31" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="T5" s="16"/>
       <c r="U5" s="17"/>
@@ -17533,7 +17535,7 @@
       <c r="Z5" s="16"/>
       <c r="AA5" s="17"/>
       <c r="AB5" s="31" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="AC5" s="16"/>
       <c r="AD5" s="17"/>
@@ -17541,7 +17543,7 @@
         <v>7</v>
       </c>
       <c r="AG5" s="36" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="AH5" s="20"/>
       <c r="AI5" s="21"/>
@@ -17556,7 +17558,7 @@
       <c r="AN5" s="16"/>
       <c r="AO5" s="17"/>
       <c r="AP5" s="31" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="AQ5" s="16"/>
       <c r="AR5" s="17"/>
@@ -17570,17 +17572,17 @@
         <v>12</v>
       </c>
       <c r="E6" s="15" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="F6" s="16"/>
       <c r="G6" s="17"/>
       <c r="H6" s="15" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="I6" s="16"/>
       <c r="J6" s="17"/>
       <c r="K6" s="15" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="L6" s="16"/>
       <c r="M6" s="17"/>
@@ -17622,17 +17624,17 @@
       <c r="B7" s="17"/>
       <c r="D7" s="7"/>
       <c r="E7" s="25" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="F7" s="16"/>
       <c r="G7" s="17"/>
       <c r="H7" s="25" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="I7" s="16"/>
       <c r="J7" s="17"/>
       <c r="K7" s="25" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="L7" s="16"/>
       <c r="M7" s="17"/>
@@ -17674,17 +17676,17 @@
       <c r="B8" s="17"/>
       <c r="D8" s="7"/>
       <c r="E8" s="15" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="F8" s="16"/>
       <c r="G8" s="17"/>
       <c r="H8" s="15" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="I8" s="16"/>
       <c r="J8" s="17"/>
       <c r="K8" s="15" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="L8" s="16"/>
       <c r="M8" s="17"/>
@@ -17722,17 +17724,17 @@
     <row r="9" spans="1:44" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="D9" s="7"/>
       <c r="E9" s="25" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="F9" s="16"/>
       <c r="G9" s="17"/>
       <c r="H9" s="25" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="I9" s="16"/>
       <c r="J9" s="17"/>
       <c r="K9" s="25" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="L9" s="16"/>
       <c r="M9" s="17"/>
@@ -17770,17 +17772,17 @@
     <row r="10" spans="1:44" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="D10" s="7"/>
       <c r="E10" s="15" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="F10" s="16"/>
       <c r="G10" s="17"/>
       <c r="H10" s="15" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="I10" s="16"/>
       <c r="J10" s="17"/>
       <c r="K10" s="15" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="L10" s="16"/>
       <c r="M10" s="17"/>
@@ -17817,7 +17819,7 @@
     </row>
     <row r="11" spans="1:44" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="3" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B11" s="3"/>
       <c r="D11" s="7"/>
@@ -17989,7 +17991,7 @@
     </row>
     <row r="15" spans="1:44" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="3" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B15" s="3"/>
       <c r="D15" s="7"/>

</xml_diff>